<commit_message>
feat(processor): add declarative table support for DOC and XLSX formats
- Implement TableBuilder for DOC/DOCX declarative table rendering as text-grid fallback
- Add TableXlsxBuilder support for XLS/XLSX with colspan and bold styling features
- Extend DocxDocumentProcessor to handle declarative TableBuilder payloads
- Enhance PoiWorkbookProcessor with declarative XLSX table insertion logic
- Update documentation with new declarative table usage examples
- Add validation and warning handling for empty or invalid declarative tables
- Introduce helper methods for cell styling, merging, and span handling in XLSX
- Refactor table anchor classes to support multiple payload types
</commit_message>
<xml_diff>
--- a/table_with_row_and_template_difficult.xlsx
+++ b/table_with_row_and_template_difficult.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="13320"/>
+    <workbookView windowHeight="14440"/>
   </bookViews>
   <sheets>
     <sheet name="Жилищная_программа" sheetId="1" r:id="rId1"/>
@@ -1569,7 +1569,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="">
       <a:dk1>

</xml_diff>